<commit_message>
added calculateoffeasbility by YBALCI
</commit_message>
<xml_diff>
--- a/2026.05.11_EKA Enerji-İstasyon proje yatırım dosyası.xlsx
+++ b/2026.05.11_EKA Enerji-İstasyon proje yatırım dosyası.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emlakasansor-my.sharepoint.com/personal/semih_eglen_ekaenerjiteknoloji_com_tr/Documents/Masaüstü/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emlakasansor-my.sharepoint.com/personal/yusuf_balci_ekaenerjiteknoloji_com_tr/Documents/Masaüstü/feasbiltynew/feasibility.v4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="700" documentId="11_AD4D0BC4A776854ACB15BCFBA654FAB6693EDF1E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB556D0D-6EB4-419E-A137-CC1EDDF31CA4}"/>
+  <xr:revisionPtr revIDLastSave="1019" documentId="11_AD4D0BC4A776854ACB15BCFBA654FAB6693EDF1E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99F8948E-420D-43CC-A5A2-F78C96F38019}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fizibilite" sheetId="1" r:id="rId1"/>
     <sheet name="Yatırım Geri Dönüş" sheetId="2" r:id="rId2"/>
+    <sheet name="Düzeltilmiş Model" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="104">
   <si>
     <t>$ Kuru</t>
   </si>
@@ -271,6 +272,84 @@
   </si>
   <si>
     <t>DEĞİŞKENLER</t>
+  </si>
+  <si>
+    <t>VARSAYIMLAR</t>
+  </si>
+  <si>
+    <t>DÜZELTİLMİŞ ÇOK YILLI FİZİBİLİTE MODELİ</t>
+  </si>
+  <si>
+    <t>Toplam Yatirim (1.yil, USD)</t>
+  </si>
+  <si>
+    <t>Yil-1 Brut Kar (USD, mevcut model)</t>
+  </si>
+  <si>
+    <t>Opex Orani (Brut Kar uzerinden)</t>
+  </si>
+  <si>
+    <t>Yillik Bakim Anlasmasi (USD)</t>
+  </si>
+  <si>
+    <t>Garanti Suresi (yil, bakim=0)</t>
+  </si>
+  <si>
+    <t>Yillik USD Enflasyonu (gelir+gider)</t>
+  </si>
+  <si>
+    <t>Iskonto Orani (NPV, USD bazli)</t>
+  </si>
+  <si>
+    <t>YIL</t>
+  </si>
+  <si>
+    <t>Iskonto Faktoru</t>
+  </si>
+  <si>
+    <t>0 (Yatirim)</t>
+  </si>
+  <si>
+    <t>SONUCLAR</t>
+  </si>
+  <si>
+    <t>IRR (10 yil, USD)</t>
+  </si>
+  <si>
+    <t>Nominal Net Kar Toplami (USD)</t>
+  </si>
+  <si>
+    <t>ESKI MODEL Geri Donus (yil)</t>
+  </si>
+  <si>
+    <t>Net Kar (opex+bakim dusulmus) + Enflasyon + NPV/IRR + Gercek basabas</t>
+  </si>
+  <si>
+    <t>Brut Kar</t>
+  </si>
+  <si>
+    <t>Opex</t>
+  </si>
+  <si>
+    <t>Bakim</t>
+  </si>
+  <si>
+    <t>Net Nakit Akisi</t>
+  </si>
+  <si>
+    <t>Bugunku Deger</t>
+  </si>
+  <si>
+    <t>Kumulatif BD</t>
+  </si>
+  <si>
+    <t>NPV (10 yil, iskontolu USD)</t>
+  </si>
+  <si>
+    <t>Kumulatif BD 10 yil sonunda (USD)</t>
+  </si>
+  <si>
+    <t>NOT: H25 negatifse yatirim 10 yilda geri donmuyor demektir.</t>
   </si>
 </sst>
 </file>
@@ -367,7 +446,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -459,6 +538,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -766,31 +849,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
       <c r="H1" s="22" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="E2" s="30" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2507,4 +2590,526 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E302985-4532-49E5-927E-161CA212957E}">
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34.77734375" customWidth="1"/>
+    <col min="2" max="8" width="15.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="31" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="32">
+        <f>Fizibilite!C8</f>
+        <v>121302.33583076244</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" s="32">
+        <f>'Yatırım Geri Dönüş'!O22</f>
+        <v>7181.3161084178055</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="33">
+        <f>Fizibilite!C29</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="32">
+        <f>Fizibilite!C31</f>
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="33">
+        <f>Fizibilite!C22</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="H14" s="31" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="32">
+        <f>-B5</f>
+        <v>-121302.33583076244</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <f t="shared" ref="G15:G25" si="0">E15*F15</f>
+        <v>-121302.33583076244</v>
+      </c>
+      <c r="H15">
+        <f>G15</f>
+        <v>-121302.33583076244</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2026</v>
+      </c>
+      <c r="B16">
+        <f>$B$6*(1+$B$10)^(1-1)</f>
+        <v>7181.3161084178055</v>
+      </c>
+      <c r="C16">
+        <f t="shared" ref="C16:C25" si="1">B16*$B$7</f>
+        <v>1436.2632216835611</v>
+      </c>
+      <c r="D16">
+        <f>IF(1&lt;=$B$9,0,$B$8*(1+$B$10)^(1-1))</f>
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <f t="shared" ref="E16:E25" si="2">B16-C16-D16</f>
+        <v>5745.0528867342446</v>
+      </c>
+      <c r="F16">
+        <f>1/(1+$B$11)^1</f>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>5222.7753515765862</v>
+      </c>
+      <c r="H16">
+        <f t="shared" ref="H16:H25" si="3">H15+G16</f>
+        <v>-116079.56047918586</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2027</v>
+      </c>
+      <c r="B17">
+        <f>$B$6*(1+$B$10)^(2-1)</f>
+        <v>7540.3819138386962</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="1"/>
+        <v>1508.0763827677392</v>
+      </c>
+      <c r="D17">
+        <f>IF(2&lt;=$B$9,0,$B$8*(1+$B$10)^(2-1))</f>
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="2"/>
+        <v>6032.3055310709569</v>
+      </c>
+      <c r="F17">
+        <f>1/(1+$B$11)^2</f>
+        <v>0.82644628099173545</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>4985.3764719594683</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="3"/>
+        <v>-111094.1840072264</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2028</v>
+      </c>
+      <c r="B18">
+        <f>$B$6*(1+$B$10)^(3-1)</f>
+        <v>7917.4010095306312</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="1"/>
+        <v>1583.4802019061262</v>
+      </c>
+      <c r="D18">
+        <f>IF(3&lt;=$B$9,0,$B$8*(1+$B$10)^(3-1))</f>
+        <v>1323</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="2"/>
+        <v>5010.920807624505</v>
+      </c>
+      <c r="F18">
+        <f>1/(1+$B$11)^3</f>
+        <v>0.75131480090157754</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>3764.7789689139772</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="3"/>
+        <v>-107329.40503831243</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2029</v>
+      </c>
+      <c r="B19">
+        <f>$B$6*(1+$B$10)^(4-1)</f>
+        <v>8313.2710600071623</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="1"/>
+        <v>1662.6542120014326</v>
+      </c>
+      <c r="D19">
+        <f>IF(4&lt;=$B$9,0,$B$8*(1+$B$10)^(4-1))</f>
+        <v>1389.15</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="2"/>
+        <v>5261.4668480057298</v>
+      </c>
+      <c r="F19">
+        <f>1/(1+$B$11)^4</f>
+        <v>0.68301345536507052</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>3593.6526521451597</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="3"/>
+        <v>-103735.75238616727</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2030</v>
+      </c>
+      <c r="B20">
+        <f>$B$6*(1+$B$10)^(5-1)</f>
+        <v>8728.934613007521</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="1"/>
+        <v>1745.7869226015043</v>
+      </c>
+      <c r="D20">
+        <f>IF(5&lt;=$B$9,0,$B$8*(1+$B$10)^(5-1))</f>
+        <v>1458.6075000000001</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="2"/>
+        <v>5524.5401904060163</v>
+      </c>
+      <c r="F20">
+        <f>1/(1+$B$11)^5</f>
+        <v>0.62092132305915493</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>3430.3048043203794</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="3"/>
+        <v>-100305.44758184689</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2031</v>
+      </c>
+      <c r="B21">
+        <f>$B$6*(1+$B$10)^(6-1)</f>
+        <v>9165.3813436578967</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="1"/>
+        <v>1833.0762687315794</v>
+      </c>
+      <c r="D21">
+        <f>IF(6&lt;=$B$9,0,$B$8*(1+$B$10)^(6-1))</f>
+        <v>1531.5378750000002</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="2"/>
+        <v>5800.7671999263175</v>
+      </c>
+      <c r="F21">
+        <f>1/(1+$B$11)^6</f>
+        <v>0.56447393005377722</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>3274.3818586694533</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="3"/>
+        <v>-97031.065723177438</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2032</v>
+      </c>
+      <c r="B22">
+        <f>$B$6*(1+$B$10)^(7-1)</f>
+        <v>9623.6504108407917</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="1"/>
+        <v>1924.7300821681583</v>
+      </c>
+      <c r="D22">
+        <f>IF(7&lt;=$B$9,0,$B$8*(1+$B$10)^(7-1))</f>
+        <v>1608.1147687499999</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="2"/>
+        <v>6090.8055599226336</v>
+      </c>
+      <c r="F22">
+        <f>1/(1+$B$11)^7</f>
+        <v>0.51315811823070645</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>3125.5463196390228</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="3"/>
+        <v>-93905.519403538419</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2033</v>
+      </c>
+      <c r="B23">
+        <f>$B$6*(1+$B$10)^(8-1)</f>
+        <v>10104.832931382833</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="1"/>
+        <v>2020.9665862765667</v>
+      </c>
+      <c r="D23">
+        <f>IF(8&lt;=$B$9,0,$B$8*(1+$B$10)^(8-1))</f>
+        <v>1688.5205071875002</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="2"/>
+        <v>6395.345837918765</v>
+      </c>
+      <c r="F23">
+        <f>1/(1+$B$11)^8</f>
+        <v>0.46650738020973315</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>2983.4760323827036</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="3"/>
+        <v>-90922.043371155713</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2034</v>
+      </c>
+      <c r="B24">
+        <f>$B$6*(1+$B$10)^(9-1)</f>
+        <v>10610.074577951973</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="1"/>
+        <v>2122.0149155903946</v>
+      </c>
+      <c r="D24">
+        <f>IF(9&lt;=$B$9,0,$B$8*(1+$B$10)^(9-1))</f>
+        <v>1772.946532546875</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="2"/>
+        <v>6715.1131298147029</v>
+      </c>
+      <c r="F24">
+        <f>1/(1+$B$11)^9</f>
+        <v>0.42409761837248466</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>2847.8634854562169</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="3"/>
+        <v>-88074.179885699501</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2035</v>
+      </c>
+      <c r="B25">
+        <f>$B$6*(1+$B$10)^(10-1)</f>
+        <v>11140.578306849571</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="1"/>
+        <v>2228.1156613699145</v>
+      </c>
+      <c r="D25">
+        <f>IF(10&lt;=$B$9,0,$B$8*(1+$B$10)^(10-1))</f>
+        <v>1861.593859174219</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="2"/>
+        <v>7050.8687863054374</v>
+      </c>
+      <c r="F25">
+        <f>1/(1+$B$11)^10</f>
+        <v>0.38554328942953148</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>2718.4151452082065</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="3"/>
+        <v>-85355.7647404913</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="31" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28">
+        <f>SUM(G15:G25)</f>
+        <v>-85355.7647404913</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="33">
+        <f>IRR(E15:E25)</f>
+        <v>-0.10822560333411024</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30">
+        <f>SUM(E16:E25)</f>
+        <v>59627.186777729308</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="34">
+        <f>'Yatırım Geri Dönüş'!Q22</f>
+        <v>16.891379518661502</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32">
+        <f>H25</f>
+        <v>-85355.7647404913</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>